<commit_message>
fix: L2 通类项扩散到 L3 children idx (v30)
用户反馈:稻谷详情页 (L3 谷物 → 稻谷) 总汞 Hg 显示 2 条重复 row。
对照 PDF 截图稻谷只有 1 条 总汞 ≤0.02。

根因:Excel 3.汞 sheet r35-r46 把 GB 标准的 1 条 L2 通类项 row (涵盖稻谷/糙米/.../小麦粉)
录入时拆成 6 条 (a1_l3 分别为 稻谷/玉米/小麦, 各自 2 污染物 row)。
v23+v29 兄弟节点探测让 row a1_l3=玉米 兄弟扩散到 idx[L3 稻谷],
row a1_l3=稻谷 自己 + row a1_l3=玉米 兄弟扩散 = idx[L3 稻谷] 总汞 2 条 (注 b 与注空, dupKey 不同不去重)。

修复:
1. Excel 3.汞 sheet 录入修正:r35/r36 改 a1_l3=空 (L2 通类项);删除 r41/r42/r45/r46 (玉米/小麦 重复)
2. 新增 v30 L2 通类项扩散:row.a1_l3 空 + path.length === 2 时,把 row 推送到 L3 children idx
   (与 v23/v29 兄弟节点探测不同: v23 是 a1_l3 row → siblings, v30 是 L2 通类项 row → children)
   仅在 a1_l3 空时触发,避免 row.a1_l3='玉米' 重复聚合。

验证:
- idx[L3 稻谷] 总汞 0.02 note=b (v30 扩散) + 甲基汞 a — (v30 扩散, 不同污染物)
- idx[L2 谷物] 5 条 row (镉 0.1 + 汞 0.02 + 甲基汞 a — + 砷 0.5 + 铬 1.0)
- v23+v29 兄弟节点探测仍正常工作: idx[L3 双孢菇]=1 / 平菇=1 / 香菇=2

涉及文件:
- data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx (3.汞 r35/r36 改 a1_l3, 删除 r41/r42/r45/r46)
- gb2762.html (新增 v30 L2 通类项扩散逻辑)
- sw.js (CACHE_BUST v30)
</commit_message>
<xml_diff>
--- a/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
+++ b/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
@@ -11964,7 +11964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K80"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="30" customWidth="1" style="23" min="1" max="1"/>
@@ -13520,11 +13520,7 @@
           <t>谷物</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>稻谷</t>
-        </is>
-      </c>
+      <c r="C35" s="4" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="inlineStr">
         <is>
@@ -13569,11 +13565,7 @@
           <t>谷物</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>稻谷</t>
-        </is>
-      </c>
+      <c r="C36" s="4" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
@@ -13791,12 +13783,12 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>谷物</t>
+          <t>谷物碾磨加工品</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>玉米</t>
+          <t>玉米粉、玉米糁(渣)</t>
         </is>
       </c>
       <c r="D41" s="4" t="n"/>
@@ -13836,15 +13828,14 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>谷物</t>
+          <t>谷物碾磨加工品</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>玉米</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="n"/>
+          <t>玉米粉、玉米糁(渣)</t>
+        </is>
+      </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
           <t>稻谷、糙米、大米(粉)、玉米、玉米粉、玉米糁(渣)、小麦、小麦粉</t>
@@ -13866,7 +13857,6 @@
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J42" s="4" t="n"/>
       <c r="K42" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -13886,7 +13876,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>玉米粉、玉米糁(渣)</t>
+          <t>小麦粉(包括食用麸皮)</t>
         </is>
       </c>
       <c r="D43" s="4" t="n"/>
@@ -13931,9 +13921,10 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>玉米粉、玉米糁(渣)</t>
-        </is>
-      </c>
+          <t>小麦粉(包括食用麸皮)</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
           <t>稻谷、糙米、大米(粉)、玉米、玉米粉、玉米糁(渣)、小麦、小麦粉</t>
@@ -13955,6 +13946,7 @@
           <t>mg/kg</t>
         </is>
       </c>
+      <c r="J44" s="4" t="n"/>
       <c r="K44" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -13964,23 +13956,19 @@
     <row r="45" ht="28" customHeight="1" s="23">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>谷物及其制品（不包括焙烤制品）</t>
+          <t>蔬菜及其制品（包括薯类，不包括食用菌）</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>谷物</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>小麦</t>
-        </is>
-      </c>
+          <t>新鲜蔬菜（未经加工的、经表面处理的、去皮或预切的、冷冻的蔬菜）</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n"/>
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>稻谷、糙米、大米(粉)、玉米、玉米粉、玉米糁(渣)、小麦、小麦粉</t>
+          <t>新鲜蔬菜</t>
         </is>
       </c>
       <c r="F45" s="12" t="inlineStr">
@@ -13990,7 +13978,7 @@
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H45" s="4" t="n"/>
@@ -14009,23 +13997,19 @@
     <row r="46" ht="28" customHeight="1" s="23">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>谷物及其制品（不包括焙烤制品）</t>
+          <t>蔬菜及其制品（包括薯类，不包括食用菌）</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>谷物</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>小麦</t>
-        </is>
-      </c>
+          <t>新鲜蔬菜（未经加工的、经表面处理的、去皮或预切的、冷冻的蔬菜）</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n"/>
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>稻谷、糙米、大米(粉)、玉米、玉米粉、玉米糁(渣)、小麦、小麦粉</t>
+          <t>新鲜蔬菜</t>
         </is>
       </c>
       <c r="F46" s="12" t="inlineStr">
@@ -14054,23 +14038,19 @@
     <row r="47" ht="28" customHeight="1" s="23">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>谷物及其制品（不包括焙烤制品）</t>
+          <t>食用菌及其制品</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>谷物碾磨加工品</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>小麦粉(包括食用麸皮)</t>
-        </is>
-      </c>
+          <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n"/>
       <c r="D47" s="4" t="n"/>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>稻谷、糙米、大米(粉)、玉米、玉米粉、玉米糁(渣)、小麦、小麦粉</t>
+          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
         </is>
       </c>
       <c r="F47" s="12" t="inlineStr">
@@ -14080,7 +14060,7 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" s="4" t="n"/>
@@ -14099,28 +14079,24 @@
     <row r="48" ht="28" customHeight="1" s="23">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>谷物及其制品（不包括焙烤制品）</t>
+          <t>食用菌及其制品</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>谷物碾磨加工品</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>小麦粉(包括食用麸皮)</t>
-        </is>
-      </c>
+          <t>食用菌制品</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n"/>
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>稻谷、糙米、大米(粉)、玉米、玉米粉、玉米糁(渣)、小麦、小麦粉</t>
+          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
         <is>
-          <t>甲基汞 a</t>
+          <t>总汞</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -14144,29 +14120,29 @@
     <row r="49" ht="28" customHeight="1" s="23">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>蔬菜及其制品（包括薯类，不包括食用菌）</t>
+          <t>食用菌及其制品</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>新鲜蔬菜（未经加工的、经表面处理的、去皮或预切的、冷冻的蔬菜）</t>
+          <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
         </is>
       </c>
       <c r="C49" s="4" t="n"/>
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>新鲜蔬菜</t>
+          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>总汞</t>
+          <t>甲基汞 a</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="H49" s="4" t="n"/>
@@ -14175,7 +14151,11 @@
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J49" s="4" t="n"/>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -14185,19 +14165,19 @@
     <row r="50" ht="28" customHeight="1" s="23">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>蔬菜及其制品（包括薯类，不包括食用菌）</t>
+          <t>食用菌及其制品</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>新鲜蔬菜（未经加工的、经表面处理的、去皮或预切的、冷冻的蔬菜）</t>
+          <t>食用菌制品</t>
         </is>
       </c>
       <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="n"/>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>新鲜蔬菜</t>
+          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
@@ -14207,7 +14187,7 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="H50" s="4" t="n"/>
@@ -14216,7 +14196,11 @@
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J50" s="4" t="n"/>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -14234,11 +14218,15 @@
           <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
         </is>
       </c>
-      <c r="C51" s="4" t="n"/>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>木耳（毛木耳,黑木耳）</t>
+        </is>
+      </c>
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
+          <t>木耳及其制品、银耳及其制品</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
@@ -14275,11 +14263,19 @@
           <t>食用菌制品</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>其他食用菌制品</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>木耳制品、银耳制品</t>
+        </is>
+      </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
+          <t>木耳及其制品、银耳及其制品</t>
         </is>
       </c>
       <c r="F52" s="12" t="inlineStr">
@@ -14316,11 +14312,15 @@
           <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n"/>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>木耳（毛木耳,黑木耳）</t>
+        </is>
+      </c>
       <c r="D53" s="4" t="n"/>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
+          <t>木耳及其制品、银耳及其制品</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
@@ -14333,7 +14333,11 @@
           <t>0.1</t>
         </is>
       </c>
-      <c r="H53" s="4" t="n"/>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>干重计</t>
+        </is>
+      </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
           <t>mg/kg</t>
@@ -14361,11 +14365,19 @@
           <t>食用菌制品</t>
         </is>
       </c>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>其他食用菌制品</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>木耳制品、银耳制品</t>
+        </is>
+      </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品(木耳及其制品、银耳及其制品除外)</t>
+          <t>木耳及其制品、银耳及其制品</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
@@ -14378,7 +14390,11 @@
           <t>0.1</t>
         </is>
       </c>
-      <c r="H54" s="4" t="n"/>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>干重计</t>
+        </is>
+      </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
           <t>mg/kg</t>
@@ -14408,7 +14424,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>木耳（毛木耳,黑木耳）</t>
+          <t>银耳</t>
         </is>
       </c>
       <c r="D55" s="4" t="n"/>
@@ -14448,19 +14464,15 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>食用菌制品</t>
+          <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>其他食用菌制品</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>木耳制品、银耳制品</t>
-        </is>
-      </c>
+          <t>银耳</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="n"/>
       <c r="E56" s="4" t="inlineStr">
         <is>
           <t>木耳及其制品、银耳及其制品</t>
@@ -14468,21 +14480,29 @@
       </c>
       <c r="F56" s="12" t="inlineStr">
         <is>
-          <t>总汞</t>
+          <t>甲基汞 a</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="n"/>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>干重计</t>
+        </is>
+      </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J56" s="4" t="n"/>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -14492,50 +14512,38 @@
     <row r="57" ht="28" customHeight="1" s="23">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品</t>
+          <t>肉及肉制品</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>木耳（毛木耳,黑木耳）</t>
-        </is>
-      </c>
+          <t>肉类(生鲜肉、冷却肉、冷冻肉等)</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="n"/>
       <c r="D57" s="4" t="n"/>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>木耳及其制品、银耳及其制品</t>
+          <t>肉类</t>
         </is>
       </c>
       <c r="F57" s="12" t="inlineStr">
         <is>
-          <t>甲基汞 a</t>
+          <t>总汞</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>干重计</t>
-        </is>
-      </c>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="inlineStr">
         <is>
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
+      <c r="J57" s="4" t="n"/>
       <c r="K57" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -14545,27 +14553,19 @@
     <row r="58" ht="28" customHeight="1" s="23">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品</t>
+          <t>肉及肉制品</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>食用菌制品</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>其他食用菌制品</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>木耳制品、银耳制品</t>
-        </is>
-      </c>
+          <t>肉类(生鲜肉、冷却肉、冷冻肉等)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="4" t="n"/>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>木耳及其制品、银耳及其制品</t>
+          <t>肉类</t>
         </is>
       </c>
       <c r="F58" s="12" t="inlineStr">
@@ -14575,24 +14575,16 @@
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>干重计</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="inlineStr">
         <is>
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
+      <c r="J58" s="4" t="n"/>
       <c r="K58" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -14602,23 +14594,19 @@
     <row r="59" ht="28" customHeight="1" s="23">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品</t>
+          <t>乳及乳制品</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>银耳</t>
-        </is>
-      </c>
+          <t>生乳</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="n"/>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>木耳及其制品、银耳及其制品</t>
+          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
         </is>
       </c>
       <c r="F59" s="12" t="inlineStr">
@@ -14628,7 +14616,7 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H59" s="4" t="n"/>
@@ -14647,23 +14635,19 @@
     <row r="60" ht="28" customHeight="1" s="23">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>食用菌及其制品</t>
+          <t>乳及乳制品</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>新鲜食用菌（未经加工的、经表面处理的、预切的、冷冻的食用菌）</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>银耳</t>
-        </is>
-      </c>
+          <t>生乳</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n"/>
       <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>木耳及其制品、银耳及其制品</t>
+          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
         </is>
       </c>
       <c r="F60" s="12" t="inlineStr">
@@ -14673,24 +14657,16 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>干重计</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="inlineStr">
         <is>
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
+      <c r="J60" s="4" t="n"/>
       <c r="K60" s="4" t="inlineStr">
         <is>
           <t>GB 5009.17</t>
@@ -14700,19 +14676,19 @@
     <row r="61" ht="28" customHeight="1" s="23">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>肉及肉制品</t>
+          <t>乳及乳制品</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>肉类(生鲜肉、冷却肉、冷冻肉等)</t>
+          <t>巴氏杀菌乳</t>
         </is>
       </c>
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>肉类</t>
+          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
         </is>
       </c>
       <c r="F61" s="12" t="inlineStr">
@@ -14722,7 +14698,7 @@
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="H61" s="4" t="n"/>
@@ -14741,19 +14717,19 @@
     <row r="62" ht="28" customHeight="1" s="23">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>肉及肉制品</t>
+          <t>乳及乳制品</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>肉类(生鲜肉、冷却肉、冷冻肉等)</t>
+          <t>巴氏杀菌乳</t>
         </is>
       </c>
       <c r="C62" s="4" t="n"/>
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>肉类</t>
+          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
@@ -14787,7 +14763,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>生乳</t>
+          <t>灭菌乳</t>
         </is>
       </c>
       <c r="C63" s="4" t="n"/>
@@ -14828,7 +14804,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>生乳</t>
+          <t>灭菌乳</t>
         </is>
       </c>
       <c r="C64" s="4" t="n"/>
@@ -14869,7 +14845,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>巴氏杀菌乳</t>
+          <t>调制乳</t>
         </is>
       </c>
       <c r="C65" s="4" t="n"/>
@@ -14910,7 +14886,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>巴氏杀菌乳</t>
+          <t>调制乳</t>
         </is>
       </c>
       <c r="C66" s="4" t="n"/>
@@ -14951,7 +14927,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>灭菌乳</t>
+          <t>发酵乳</t>
         </is>
       </c>
       <c r="C67" s="4" t="n"/>
@@ -14992,7 +14968,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>灭菌乳</t>
+          <t>发酵乳</t>
         </is>
       </c>
       <c r="C68" s="4" t="n"/>
@@ -15028,19 +15004,19 @@
     <row r="69" ht="28" customHeight="1" s="23">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>乳及乳制品</t>
+          <t>蛋及蛋制品</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>调制乳</t>
+          <t>鲜蛋</t>
         </is>
       </c>
       <c r="C69" s="4" t="n"/>
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
+          <t>鲜蛋</t>
         </is>
       </c>
       <c r="F69" s="12" t="inlineStr">
@@ -15050,7 +15026,7 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="H69" s="4" t="n"/>
@@ -15069,19 +15045,19 @@
     <row r="70" ht="28" customHeight="1" s="23">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>乳及乳制品</t>
+          <t>蛋及蛋制品</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>调制乳</t>
+          <t>鲜蛋</t>
         </is>
       </c>
       <c r="C70" s="4" t="n"/>
       <c r="D70" s="4" t="n"/>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
+          <t>鲜蛋</t>
         </is>
       </c>
       <c r="F70" s="12" t="inlineStr">
@@ -15110,19 +15086,19 @@
     <row r="71" ht="28" customHeight="1" s="23">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>乳及乳制品</t>
+          <t>调味品</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>发酵乳</t>
+          <t>食用盐</t>
         </is>
       </c>
       <c r="C71" s="4" t="n"/>
       <c r="D71" s="4" t="n"/>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
+          <t>食用盐</t>
         </is>
       </c>
       <c r="F71" s="12" t="inlineStr">
@@ -15132,7 +15108,7 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="H71" s="4" t="n"/>
@@ -15151,19 +15127,19 @@
     <row r="72" ht="28" customHeight="1" s="23">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>乳及乳制品</t>
+          <t>调味品</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>发酵乳</t>
+          <t>食用盐</t>
         </is>
       </c>
       <c r="C72" s="4" t="n"/>
       <c r="D72" s="4" t="n"/>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>生乳、巴氏杀菌乳、灭菌乳、调制乳、发酵乳</t>
+          <t>食用盐</t>
         </is>
       </c>
       <c r="F72" s="12" t="inlineStr">
@@ -15192,19 +15168,23 @@
     <row r="73" ht="28" customHeight="1" s="23">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>蛋及蛋制品</t>
+          <t>饮料类</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>鲜蛋</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="n"/>
+          <t>包装饮用水</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>饮用天然矿泉水</t>
+        </is>
+      </c>
       <c r="D73" s="4" t="n"/>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>鲜蛋</t>
+          <t>饮用天然矿泉水</t>
         </is>
       </c>
       <c r="F73" s="12" t="inlineStr">
@@ -15214,38 +15194,42 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>mg/kg</t>
+          <t>mg/L</t>
         </is>
       </c>
       <c r="J73" s="4" t="n"/>
       <c r="K73" s="4" t="inlineStr">
         <is>
-          <t>GB 5009.17</t>
+          <t>GB 8538</t>
         </is>
       </c>
     </row>
     <row r="74" ht="28" customHeight="1" s="23">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>蛋及蛋制品</t>
+          <t>饮料类</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>鲜蛋</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="n"/>
+          <t>包装饮用水</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>饮用天然矿泉水</t>
+        </is>
+      </c>
       <c r="D74" s="4" t="n"/>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>鲜蛋</t>
+          <t>饮用天然矿泉水</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
@@ -15261,32 +15245,36 @@
       <c r="H74" s="4" t="n"/>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>mg/kg</t>
+          <t>mg/L</t>
         </is>
       </c>
       <c r="J74" s="4" t="n"/>
       <c r="K74" s="4" t="inlineStr">
         <is>
-          <t>GB 5009.17</t>
+          <t>GB 8538</t>
         </is>
       </c>
     </row>
     <row r="75" ht="28" customHeight="1" s="23">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>调味品</t>
+          <t>特殊膳食用食品</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>食用盐</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="n"/>
+          <t>婴幼儿辅助食品</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>婴幼儿罐装辅助食品</t>
+        </is>
+      </c>
       <c r="D75" s="4" t="n"/>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>食用盐</t>
+          <t>婴幼儿罐装辅助食品</t>
         </is>
       </c>
       <c r="F75" s="12" t="inlineStr">
@@ -15296,7 +15284,7 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="H75" s="4" t="n"/>
@@ -15315,19 +15303,23 @@
     <row r="76" ht="28" customHeight="1" s="23">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>调味品</t>
+          <t>特殊膳食用食品</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>食用盐</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="n"/>
+          <t>婴幼儿辅助食品</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>婴幼儿罐装辅助食品</t>
+        </is>
+      </c>
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>食用盐</t>
+          <t>婴幼儿罐装辅助食品</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
@@ -15353,186 +15345,10 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="28" customHeight="1" s="23">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>饮料类</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>包装饮用水</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>饮用天然矿泉水</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="n"/>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>饮用天然矿泉水</t>
-        </is>
-      </c>
-      <c r="F77" s="12" t="inlineStr">
-        <is>
-          <t>总汞</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>0.001</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="n"/>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>mg/L</t>
-        </is>
-      </c>
-      <c r="J77" s="4" t="n"/>
-      <c r="K77" s="4" t="inlineStr">
-        <is>
-          <t>GB 8538</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="28" customHeight="1" s="23">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>饮料类</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>包装饮用水</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>饮用天然矿泉水</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="n"/>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>饮用天然矿泉水</t>
-        </is>
-      </c>
-      <c r="F78" s="12" t="inlineStr">
-        <is>
-          <t>甲基汞 a</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="4" t="n"/>
-      <c r="I78" s="4" t="inlineStr">
-        <is>
-          <t>mg/L</t>
-        </is>
-      </c>
-      <c r="J78" s="4" t="n"/>
-      <c r="K78" s="4" t="inlineStr">
-        <is>
-          <t>GB 8538</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="28" customHeight="1" s="23">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>特殊膳食用食品</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿辅助食品</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿罐装辅助食品</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="n"/>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿罐装辅助食品</t>
-        </is>
-      </c>
-      <c r="F79" s="12" t="inlineStr">
-        <is>
-          <t>总汞</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="n"/>
-      <c r="I79" s="4" t="inlineStr">
-        <is>
-          <t>mg/kg</t>
-        </is>
-      </c>
-      <c r="J79" s="4" t="n"/>
-      <c r="K79" s="4" t="inlineStr">
-        <is>
-          <t>GB 5009.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="28" customHeight="1" s="23">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>特殊膳食用食品</t>
-        </is>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿辅助食品</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿罐装辅助食品</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="n"/>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿罐装辅助食品</t>
-        </is>
-      </c>
-      <c r="F80" s="12" t="inlineStr">
-        <is>
-          <t>甲基汞 a</t>
-        </is>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H80" s="4" t="n"/>
-      <c r="I80" s="4" t="inlineStr">
-        <is>
-          <t>mg/kg</t>
-        </is>
-      </c>
-      <c r="J80" s="4" t="n"/>
-      <c r="K80" s="4" t="inlineStr">
-        <is>
-          <t>GB 5009.17</t>
-        </is>
-      </c>
-    </row>
+    <row r="77" ht="28" customHeight="1" s="23"/>
+    <row r="78" ht="28" customHeight="1" s="23"/>
+    <row r="79" ht="28" customHeight="1" s="23"/>
+    <row r="80" ht="28" customHeight="1" s="23"/>
   </sheetData>
   <autoFilter ref="A4:K80"/>
   <mergeCells count="1">
@@ -18702,82 +18518,82 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="0" t="inlineStr">
         <is>
           <t>谷物及其制品（不包括焙烤制品）</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="0" t="inlineStr">
         <is>
           <t>谷物</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr">
+      <c r="C75" s="0" t="inlineStr"/>
+      <c r="D75" s="0" t="inlineStr"/>
+      <c r="E75" s="0" t="inlineStr">
         <is>
           <t>谷物(稻谷除外)</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="0" t="inlineStr">
         <is>
           <t>无机砷 a</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G75" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>mg/kg</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr">
+      <c r="H75" s="0" t="inlineStr"/>
+      <c r="I75" s="0" t="inlineStr">
+        <is>
+          <t>mg/kg</t>
+        </is>
+      </c>
+      <c r="J75" s="0" t="inlineStr"/>
+      <c r="K75" s="0" t="inlineStr">
         <is>
           <t>GB 5009.11</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="0" t="inlineStr">
         <is>
           <t>谷物及其制品（不包括焙烤制品）</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="0" t="inlineStr">
         <is>
           <t>谷物碾磨加工品</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
+      <c r="C76" s="0" t="inlineStr"/>
+      <c r="D76" s="0" t="inlineStr"/>
+      <c r="E76" s="0" t="inlineStr">
         <is>
           <t>谷物碾磨加工品[糙米、大米(粉)除外]</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="0" t="inlineStr">
         <is>
           <t>无机砷 a</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G76" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>mg/kg</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr">
+      <c r="H76" s="0" t="inlineStr"/>
+      <c r="I76" s="0" t="inlineStr">
+        <is>
+          <t>mg/kg</t>
+        </is>
+      </c>
+      <c r="J76" s="0" t="inlineStr"/>
+      <c r="K76" s="0" t="inlineStr">
         <is>
           <t>GB 5009.11</t>
         </is>

</xml_diff>

<commit_message>
fix: v59 撤销 v36 L1 通类项扩散 + 修复酒类 R78/R79 food 字段
撤销原因: 用户反馈 L2 子页(如配制酒)显示 L1 通类项 row 是错误的。
  - L1 通类项是 PDF 表头限量,只应在 L1 详情页展示
  - L2 子页只展示 L2/L3 专属 row
  - L2 配制酒 PDF 中无独立限量行 → idx 应为 0
  - L2 蒸馏酒/发酵酒 PDF 中有 L3 白酒/黄酒 专属 → idx 显示对应 row

修复酒类 xlsx 数据:
- R78: a1_l3=None, food='白酒'(原 '白酒、黄酒'), note='仅限白酒'
- R79: a1_l3=None, food='黄酒'(原 '白酒、黄酒'), note='仅限黄酒'

撤销后状态 (PDF 正确版):
- L1 酒类: 1 (0.2 白酒黄酒除外)
- L2 蒸馏酒: 1 (0.5 白酒 仅限白酒)
- L2 配制酒: 0 (PDF 无独立限量)
- L2 发酵酒: 1 (0.5 黄酒 仅限黄酒)

副作用: L2 食糖/乳糖/淀粉糖 等无自己 row 的 L2 子页显示 0 (符合 PDF)。
verify_idx.py 同步撤销 v36。
</commit_message>
<xml_diff>
--- a/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
+++ b/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
@@ -6432,7 +6432,7 @@
       <c r="D78" s="19" t="n"/>
       <c r="E78" s="19" t="inlineStr">
         <is>
-          <t>白酒、黄酒</t>
+          <t>白酒</t>
         </is>
       </c>
       <c r="F78" s="19" t="inlineStr">
@@ -6451,7 +6451,11 @@
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J78" s="19" t="n"/>
+      <c r="J78" s="19" t="inlineStr">
+        <is>
+          <t>仅限白酒</t>
+        </is>
+      </c>
       <c r="K78" s="19" t="inlineStr">
         <is>
           <t>GB 5009.12</t>
@@ -6477,7 +6481,7 @@
       <c r="D79" s="19" t="n"/>
       <c r="E79" s="19" t="inlineStr">
         <is>
-          <t>白酒、黄酒</t>
+          <t>黄酒</t>
         </is>
       </c>
       <c r="F79" s="19" t="inlineStr">
@@ -6496,7 +6500,11 @@
           <t>mg/kg</t>
         </is>
       </c>
-      <c r="J79" s="19" t="n"/>
+      <c r="J79" s="19" t="inlineStr">
+        <is>
+          <t>仅限黄酒</t>
+        </is>
+      </c>
       <c r="K79" s="19" t="inlineStr">
         <is>
           <t>GB 5009.12</t>

</xml_diff>

<commit_message>
fix: v60 锡 R3 L1 改为空 + renderLimitTable row 单位/方法优先
- xlsx 5.锡 R3: a1_l1='饮料类' → '', 用户反馈锡 row 不需在 L1 饮料类下体现
- gb2762.html renderLimitTable (line 1522-1552): unit/method 优先用 row 自身字段 (it.unit/it.inspection_method) 而非整表默认 (it._unit/it._inspection_method)
- 修复 L2 包装饮用水 镉/砷/亚硝酸盐 误显示 mg/kg+GB 5009.x 整表默认
- renderContamRow (line 1937-1960) 同样的 it.inspection_method 优先
- bump CACHE_BUST v59 → v60 (sw.js + gb2762.html 4处)
</commit_message>
<xml_diff>
--- a/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
+++ b/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
@@ -15994,11 +15994,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>饮料类</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="4" t="n"/>

</xml_diff>

<commit_message>
fix: v64 锡表所有 row a1_l1/a1_l2/a1_l3/a1_l4 全部清空
用户反馈: '所有的西医(锡)只在表第一个分类当中, 食品当中体现到, 其他的各级分类不体现'

问题根因: v62 commit (100ae7d) 在修复可可制品时, 错误地从 v61 之前的备份恢复了 xlsx,
导致锡 R0/R1 (婴幼儿辅助食品 50 / 婴儿配方食品 50) 和 R2 (食品(...) 250) 的 a1_l1/a1_l2 又挂回原 A.1 分类。
v61 (2be270a) 已经把这 3 个 row 的 a1_l1/a1_l2 清空。

修复:
xlsx 5.锡 sheet row 5-8 a1_l1/a1_l2/a1_l3/a1_l4 全部清空:
- sheet row 5: 婴幼儿辅助食品 50 mg/kg (清空, 不挂 L2 婴幼儿辅助食品)
- sheet row 6: 婴儿配方食品... 50 mg/kg (清空, 不挂 L2 婴幼儿配方食品)
- sheet row 7: 食品(饮料类、婴幼儿配方食品、婴幼儿辅助食品除外) 250 mg/kg (清空)
- sheet row 8: 饮料类 150 mg/kg (v60 已清空, 保持)

verify_idx 验证:
- L2 婴幼儿配方食品: 命中 2 (铅 + 亚硝酸盐, 无锡) ✓
- L2 婴幼儿辅助食品: 命中 2 (铅 + 亚硝酸盐, 无锡) ✓
- L1 饮料类: 命中 1 (铅, 无锡) ✓

锡所有 row 现在只在污染物查询'锡' tab 显示, 不在 A.1 分类树任何节点显示。

bump CACHE_BUST v63 → v64 (sw.js + gb2762.html 4处)
</commit_message>
<xml_diff>
--- a/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
+++ b/data/gb2762/_gb2762_2025_12项污染物_v6_synced.xlsx
@@ -15992,16 +15992,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>特殊膳食用食品</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿辅助食品</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="inlineStr">
@@ -16037,16 +16029,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>特殊膳食用食品</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>婴幼儿配方食品</t>
-        </is>
-      </c>
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="inlineStr">
@@ -16082,11 +16066,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" s="23">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>食品</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>

</xml_diff>